<commit_message>
Change the joining link for session 51
Session 51, Digital Forensics and Media Authenticity (Tuesday 10:00-11:12, chair
Bojjapalli Archana), now meets at https://meet.google.com/mdt-kosz-fed in place of
https://meet.google.com/kwp-pqrs-rmb. The session 51 chair sheet is regenerated with
the new link. Its six papers' authors are being told directly.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/programme/chair-sheets/S51.xlsx
+++ b/programme/chair-sheets/S51.xlsx
@@ -58,7 +58,7 @@
     <t xml:space="preserve">Joining link</t>
   </si>
   <si>
-    <t xml:space="preserve">https://meet.google.com/kwp-pqrs-rmb</t>
+    <t xml:space="preserve">https://meet.google.com/mdt-kosz-fed</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -972,7 +972,7 @@
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="12" t="n">
-        <f aca="false">COUNTA(C11:C16)</f>
+        <f aca="false">COUNTA(C11:C16)-COUNTIF(E11:E16,"Moved")</f>
         <v>6</v>
       </c>
     </row>

</xml_diff>